<commit_message>
Add advanced WebP conversion UI and backend
Revamp webpmaker: replace the simple upload form with a richer template that shows conversion results, errors, a download link and client-side JS to toggle between conversion modes. Implement robust server-side image handling in webpmaker/app.py: EXIF orientation normalization, image validation (verify+load), secure filenames, UUID-based unique outputs, two conversion strategies (target quality and iterative max-size reduction), and safer directory creation. Produce ZIP archives of converted files and render the page with error messages and the download URL instead of redirecting. Also add many binary assets (uploads and generated WebP/ZIP files), a SQLite instance file, and update processed_data.xlsx; compiled .pyc files changed as a result of code updates.
</commit_message>
<xml_diff>
--- a/processed_data.xlsx
+++ b/processed_data.xlsx
@@ -425,670 +425,1363 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Család és szülők</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>6743</v>
+          <t>Műfajok</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Rendelés bejövő|menny.</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Rendelés bejövő|érték</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Család és szülők</t>
+          <t>Ajándékkártya</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>399</v>
       </c>
       <c r="C2" t="n">
-        <v>10629</v>
+        <v>3979000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DVD Filmek</t>
+          <t>Albumok</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>114</v>
       </c>
       <c r="C3" t="n">
-        <v>16479</v>
+        <v>585970</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Egyéb termékek</t>
+          <t>Blu-ray filmek</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="C4" t="n">
-        <v>6743</v>
+        <v>392299</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Erotikus</t>
+          <t>CD</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>137889</v>
+        <v>30857</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ezotéria</t>
+          <t>Család és szülők</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>2254</v>
       </c>
       <c r="C6" t="n">
-        <v>164524</v>
+        <v>6743279.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fantasy</t>
+          <t>DVD Filmek</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>249</v>
       </c>
       <c r="C7" t="n">
-        <v>208536</v>
+        <v>445843</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gasztronómia</t>
+          <t>Diafilm</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>427</v>
       </c>
       <c r="C8" t="n">
-        <v>76563</v>
+        <v>792797</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gazdasági, közéleti, politikai</t>
+          <t>Dráma</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="C9" t="n">
-        <v>17985</v>
+        <v>483380</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Gyerekkönyvek</t>
+          <t>Egyéb termékek</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="C10" t="n">
-        <v>735647</v>
+        <v>1330453</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Gyereknevelés</t>
+          <t>Erotikus</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>4874</v>
       </c>
       <c r="C11" t="n">
-        <v>12728</v>
+        <v>18843845</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hangoskönyv</t>
+          <t>Ezotéria</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22</v>
+        <v>18738</v>
       </c>
       <c r="C12" t="n">
-        <v>54893</v>
+        <v>61942331</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hobby, szabadidő</t>
+          <t>Fantasy</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12</v>
+        <v>16067</v>
       </c>
       <c r="C13" t="n">
-        <v>29587</v>
+        <v>73334200.90000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Horror</t>
+          <t>Filozófia</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>255</v>
       </c>
       <c r="C14" t="n">
-        <v>3735</v>
+        <v>846305</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Humor</t>
+          <t>Gasztronómia</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>4534</v>
       </c>
       <c r="C15" t="n">
-        <v>6898</v>
+        <v>15626042</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Idegen nyelvű</t>
+          <t>Gazdasági, közéleti, politikai</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>755</v>
       </c>
       <c r="C16" t="n">
-        <v>3893</v>
+        <v>2746875</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ifjúsági</t>
+          <t>Gyerek</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>86</v>
+        <v>129</v>
       </c>
       <c r="C17" t="n">
-        <v>232410</v>
+        <v>297024</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ismeretterjesztő</t>
+          <t>Gyerekkönyvek</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>18</v>
+        <v>85097</v>
       </c>
       <c r="C18" t="n">
-        <v>48487</v>
+        <v>208084412.2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Kalandregények</t>
+          <t>Gyereknevelés</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>536</v>
       </c>
       <c r="C19" t="n">
-        <v>8391</v>
+        <v>1602473</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Kert, ház, otthon</t>
+          <t>Hangoskönyv</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>121</v>
       </c>
       <c r="C20" t="n">
-        <v>2625</v>
+        <v>310823</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Krimi</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="C21" t="n">
-        <v>34590</v>
+        <v>233115</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kultúrtörténet</t>
+          <t>Hobby, szabadidő</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1615</v>
       </c>
       <c r="C22" t="n">
-        <v>6150</v>
+        <v>5092209</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Kártyák</t>
+          <t>Horror</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>14</v>
+        <v>2493</v>
       </c>
       <c r="C23" t="n">
-        <v>97803</v>
+        <v>9753362</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Képregények</t>
+          <t>Humor</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>1109</v>
       </c>
       <c r="C24" t="n">
-        <v>2246</v>
+        <v>2308578</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mesekönyv</t>
+          <t>Idegen nyelvű</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>39</v>
+        <v>246</v>
       </c>
       <c r="C25" t="n">
-        <v>106731</v>
+        <v>840217</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Művészet</t>
+          <t>Ifjúsági</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>19575</v>
       </c>
       <c r="C26" t="n">
-        <v>6859</v>
+        <v>64695082</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nyelvkönyv, szótár</t>
+          <t>Ismeretterjesztő</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>7</v>
+        <v>6555</v>
       </c>
       <c r="C27" t="n">
-        <v>24377</v>
+        <v>24184377.6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pszichológia</t>
+          <t>Kalandregények</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>19</v>
+        <v>524</v>
       </c>
       <c r="C28" t="n">
-        <v>66536</v>
+        <v>2061075</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Párkapcsolat, szerelem</t>
+          <t>Karácsony</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>197</v>
       </c>
       <c r="C29" t="n">
-        <v>3368</v>
+        <v>503391</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Regény</t>
+          <t>Kert, ház, otthon</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>27</v>
+        <v>640</v>
       </c>
       <c r="C30" t="n">
-        <v>90263</v>
+        <v>2086159</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Romantikus</t>
+          <t>Krimi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>59</v>
+        <v>10239</v>
       </c>
       <c r="C31" t="n">
-        <v>227557</v>
+        <v>40458391</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Science fiction</t>
+          <t>Kultúrtörténet</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>135</v>
       </c>
       <c r="C32" t="n">
-        <v>11363</v>
+        <v>492869</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Kártyák</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>9</v>
+        <v>2519</v>
       </c>
       <c r="C33" t="n">
-        <v>37068</v>
+        <v>12486389</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Szakkönyvek</t>
+          <t>Képregények</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2134</v>
       </c>
       <c r="C34" t="n">
-        <v>3713</v>
+        <v>7964163</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Szakácskönyv</t>
+          <t>Könyvcsomagok</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>6</v>
+        <v>1652</v>
       </c>
       <c r="C35" t="n">
-        <v>19158</v>
+        <v>28106764</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Szépirodalom</t>
+          <t>Lexikon, enciklopédia</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C36" t="n">
-        <v>151165</v>
+        <v>196500</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Szórakoztató irodalom</t>
+          <t>Mesekönyv</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>180</v>
+        <v>25950</v>
       </c>
       <c r="C37" t="n">
-        <v>916566</v>
+        <v>63488846.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Tankönyvek, segédkönyvek</t>
+          <t>Művészet</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>204</v>
+        <v>301</v>
       </c>
       <c r="C38" t="n">
-        <v>420250</v>
+        <v>1270296</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Thriller</t>
+          <t>Naptárak</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="C39" t="n">
-        <v>11513</v>
+        <v>146430</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tudományos könyvek</t>
+          <t>Nyelvkönyv, szótár</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4</v>
+        <v>867</v>
       </c>
       <c r="C40" t="n">
-        <v>14579</v>
+        <v>3032117</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Társadalomtudomány</t>
+          <t>Nőknek</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C41" t="n">
-        <v>49368</v>
+        <v>86450.60000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Társasjátékok</t>
+          <t>Outlet</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3</v>
+        <v>86021</v>
       </c>
       <c r="C42" t="n">
-        <v>14470</v>
+        <v>291307455.84</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Térképek</t>
+          <t>Papír, írószer</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C43" t="n">
-        <v>14215</v>
+        <v>108292</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Történelmi</t>
+          <t>Paranormális</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C44" t="n">
-        <v>19095</v>
+        <v>32939</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Utazás</t>
+          <t>Pszichológia</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>3097</v>
       </c>
       <c r="C45" t="n">
-        <v>2618</v>
+        <v>9133841</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vallás, mitológia</t>
+          <t>Párkapcsolat, szerelem</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>975</v>
       </c>
       <c r="C46" t="n">
-        <v>6188</v>
+        <v>2841326</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Vegyes</t>
+          <t>Regény</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>7917</v>
       </c>
       <c r="C47" t="n">
-        <v>6750</v>
+        <v>23829924</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Young Adult</t>
+          <t>Romantikus</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>9703</v>
       </c>
       <c r="C48" t="n">
-        <v>8623</v>
+        <v>35206183.5</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Életmód</t>
+          <t>Ruházat</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>82172</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Életrajz</t>
+          <t>Science fiction</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>10</v>
+        <v>16074</v>
       </c>
       <c r="C50" t="n">
-        <v>55736</v>
+        <v>69449982</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1491</v>
+      </c>
+      <c r="C51" t="n">
+        <v>6365236</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Szakkönyvek</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>285</v>
+      </c>
+      <c r="C52" t="n">
+        <v>999283</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Szakácskönyv</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1191</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3953510</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Szépirodalom</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>12115</v>
+      </c>
+      <c r="C54" t="n">
+        <v>42591297.5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Szórakoztató irodalom</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>30005</v>
+      </c>
+      <c r="C55" t="n">
+        <v>124174103.84</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tankönyvek, segédkönyvek</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>4519</v>
+      </c>
+      <c r="C56" t="n">
+        <v>9410616</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Thriller</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>7573</v>
+      </c>
+      <c r="C57" t="n">
+        <v>24083118</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Tudományos könyvek</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1776</v>
+      </c>
+      <c r="C58" t="n">
+        <v>6605243</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Társadalomtudomány</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2789</v>
+      </c>
+      <c r="C59" t="n">
+        <v>9932521</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Társasjátékok</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2516</v>
+      </c>
+      <c r="C60" t="n">
+        <v>10700215</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Táskák</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>10</v>
+      </c>
+      <c r="C61" t="n">
+        <v>13177</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Térképek</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>112</v>
+      </c>
+      <c r="C62" t="n">
+        <v>433946</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Történelmi</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3088</v>
+      </c>
+      <c r="C63" t="n">
+        <v>9307512</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Utazás</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>453</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1964368</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Vallás, mitológia</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>913</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2545948</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Vegyes</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>24148</v>
+      </c>
+      <c r="C66" t="n">
+        <v>44291220</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Young Adult</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1669</v>
+      </c>
+      <c r="C67" t="n">
+        <v>8650153</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>e-eCsalád gyermek</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>65</v>
+      </c>
+      <c r="C68" t="n">
+        <v>180220</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>e-eEgyéb</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>141</v>
+      </c>
+      <c r="C69" t="n">
+        <v>405576</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>e-eEgészség életmód</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>203</v>
+      </c>
+      <c r="C70" t="n">
+        <v>587955</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>e-eEzotéria</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>335</v>
+      </c>
+      <c r="C71" t="n">
+        <v>798728</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>e-eFantasy</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>187</v>
+      </c>
+      <c r="C72" t="n">
+        <v>808974</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>e-eGasztronómia</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>16</v>
+      </c>
+      <c r="C73" t="n">
+        <v>45531</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>e-eGyermek és ifjúsági irodalom</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>119</v>
+      </c>
+      <c r="C74" t="n">
+        <v>244464</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>e-eHobbi szabadidő</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" t="n">
+        <v>4370</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>e-eIdegennyelvű</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>32</v>
+      </c>
+      <c r="C76" t="n">
+        <v>27734</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>e-eKrimi és thriller</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>377</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1245823</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>e-eMűvészet média</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" t="n">
+        <v>5508</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>e-ePszichológia, önfejlesztés</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>288</v>
+      </c>
+      <c r="C79" t="n">
+        <v>906392</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>e-eRomantika erotika</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>534</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1876203</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>e-eSci fi</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>288</v>
+      </c>
+      <c r="C81" t="n">
+        <v>934384</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>e-eSport</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>5</v>
+      </c>
+      <c r="C82" t="n">
+        <v>14745</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>e-eSzámítástechnika</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>15</v>
+      </c>
+      <c r="C83" t="n">
+        <v>56549</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>e-eSzépirodalom</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>200</v>
+      </c>
+      <c r="C84" t="n">
+        <v>458466</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>e-eSzórakoztató irodalom</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>322</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1021547</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>e-eTermészettudomány</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>10</v>
+      </c>
+      <c r="C86" t="n">
+        <v>35607</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>e-eTársadalomtudomány</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>194</v>
+      </c>
+      <c r="C87" t="n">
+        <v>475484</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>e-eTörténettudomány</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>20</v>
+      </c>
+      <c r="C88" t="n">
+        <v>52179</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>e-eVallás</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>9</v>
+      </c>
+      <c r="C89" t="n">
+        <v>28040</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>e-eÉletrajzok önéletrajzok</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>8</v>
+      </c>
+      <c r="C90" t="n">
+        <v>25943</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>e-eÜzlet gazdaság</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>21</v>
+      </c>
+      <c r="C91" t="n">
+        <v>50948</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>e-könyv</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>4</v>
+      </c>
+      <c r="C92" t="n">
+        <v>8636</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>eCsalád gyermek</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>eEzotéria</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>8</v>
+      </c>
+      <c r="C94" t="n">
+        <v>16458</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>eFantasy</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>3</v>
+      </c>
+      <c r="C95" t="n">
+        <v>5940</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ePszichológia</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>5</v>
+      </c>
+      <c r="C96" t="n">
+        <v>7665</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ePszichológia, önfejlesztés</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>3</v>
+      </c>
+      <c r="C97" t="n">
+        <v>8523</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>eSci fi</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>13</v>
+      </c>
+      <c r="C98" t="n">
+        <v>25641</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>eSzórakoztató irodalom</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" t="n">
+        <v>2754</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>eeÁllattartás</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>8</v>
+      </c>
+      <c r="C100" t="n">
+        <v>24028</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>könyv</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>0</v>
+      </c>
+      <c r="C101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Életmód</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>9530</v>
+      </c>
+      <c r="C102" t="n">
+        <v>38158284.6</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Életrajz</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>1664</v>
+      </c>
+      <c r="C103" t="n">
+        <v>7094808.5</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>Önfejlesztő könyvek</t>
         </is>
       </c>
-      <c r="B51" t="n">
-        <v>15</v>
-      </c>
-      <c r="C51" t="n">
-        <v>47771</v>
+      <c r="B104" t="n">
+        <v>6680</v>
+      </c>
+      <c r="C104" t="n">
+        <v>18817353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>